<commit_message>
Modify gantt chart column and row widths
</commit_message>
<xml_diff>
--- a/docs/diagrams/gantt_initial.xlsx
+++ b/docs/diagrams/gantt_initial.xlsx
@@ -1,20 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26227"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\andre\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\ASU Engineering\Semesters\Senior I\Spring 26\CSE 352\Project\Marketplace\docs\diagrams\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF4F1243-32D7-4071-B057-D9DA99956AFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{368B3983-253F-4421-9557-176360953044}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-104" yWindow="-104" windowWidth="22326" windowHeight="12050" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Gantt Chart" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Gantt Chart'!$A$1:$AC$73</definedName>
+  </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
@@ -892,18 +895,13 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
@@ -937,13 +935,7 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -961,15 +953,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="14" fillId="13" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" indent="1"/>
     </xf>
@@ -977,24 +960,11 @@
     <xf numFmtId="0" fontId="14" fillId="8" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="16" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="19" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="17" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="14" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1003,6 +973,39 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="22" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="22" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="23" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1318,206 +1321,228 @@
   <dimension ref="A1:AD73"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="50" customWidth="1"/>
-    <col min="2" max="2" width="11" customWidth="1"/>
-    <col min="3" max="29" width="3.21875" customWidth="1"/>
+    <col min="1" max="1" width="45.8984375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.3984375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.19921875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="2.296875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="2.5" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.8984375" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="2.5" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="5.59765625" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="2.5" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="5.59765625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="2.5" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="1.796875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="5.59765625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="1.8984375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="2.09765625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="10.796875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="2.3984375" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="1.8984375" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="6.69921875" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="1.8984375" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="2.296875" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="4.69921875" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="2.296875" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="2.3984375" bestFit="1" customWidth="1"/>
+    <col min="27" max="29" width="2.296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:29" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="34" t="s">
+    <row r="1" spans="1:29" ht="28.1" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="54" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="35"/>
-      <c r="C1" s="35"/>
-      <c r="D1" s="35"/>
-      <c r="E1" s="35"/>
-      <c r="F1" s="35"/>
-      <c r="G1" s="35"/>
-      <c r="H1" s="35"/>
-      <c r="I1" s="35"/>
-      <c r="J1" s="35"/>
-      <c r="K1" s="35"/>
-      <c r="L1" s="35"/>
-      <c r="M1" s="35"/>
-      <c r="N1" s="35"/>
-      <c r="O1" s="35"/>
-      <c r="P1" s="35"/>
-      <c r="Q1" s="35"/>
-      <c r="R1" s="35"/>
-      <c r="S1" s="35"/>
-      <c r="T1" s="35"/>
-      <c r="U1" s="35"/>
-      <c r="V1" s="35"/>
-      <c r="W1" s="35"/>
-      <c r="X1" s="35"/>
-      <c r="Y1" s="35"/>
-      <c r="Z1" s="35"/>
-      <c r="AA1" s="35"/>
-      <c r="AB1" s="35"/>
-      <c r="AC1" s="36"/>
+      <c r="B1" s="55"/>
+      <c r="C1" s="55"/>
+      <c r="D1" s="55"/>
+      <c r="E1" s="55"/>
+      <c r="F1" s="55"/>
+      <c r="G1" s="55"/>
+      <c r="H1" s="55"/>
+      <c r="I1" s="55"/>
+      <c r="J1" s="55"/>
+      <c r="K1" s="55"/>
+      <c r="L1" s="55"/>
+      <c r="M1" s="55"/>
+      <c r="N1" s="55"/>
+      <c r="O1" s="55"/>
+      <c r="P1" s="55"/>
+      <c r="Q1" s="55"/>
+      <c r="R1" s="55"/>
+      <c r="S1" s="55"/>
+      <c r="T1" s="55"/>
+      <c r="U1" s="55"/>
+      <c r="V1" s="55"/>
+      <c r="W1" s="55"/>
+      <c r="X1" s="55"/>
+      <c r="Y1" s="55"/>
+      <c r="Z1" s="55"/>
+      <c r="AA1" s="55"/>
+      <c r="AB1" s="55"/>
+      <c r="AC1" s="56"/>
     </row>
     <row r="2" spans="1:29" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="37" t="s">
+      <c r="A2" s="30" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="38" t="s">
+      <c r="B2" s="31" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="39" t="s">
+      <c r="C2" s="32" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="40" t="s">
+      <c r="D2" s="33" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="40" t="s">
+      <c r="E2" s="33" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="40" t="s">
+      <c r="F2" s="33" t="s">
         <v>6</v>
       </c>
-      <c r="G2" s="40" t="s">
+      <c r="G2" s="33" t="s">
         <v>7</v>
       </c>
-      <c r="H2" s="40" t="s">
+      <c r="H2" s="33" t="s">
         <v>8</v>
       </c>
-      <c r="I2" s="40" t="s">
+      <c r="I2" s="33" t="s">
         <v>9</v>
       </c>
-      <c r="J2" s="40" t="s">
+      <c r="J2" s="33" t="s">
         <v>10</v>
       </c>
-      <c r="K2" s="40" t="s">
+      <c r="K2" s="33" t="s">
         <v>11</v>
       </c>
-      <c r="L2" s="40" t="s">
+      <c r="L2" s="33" t="s">
         <v>12</v>
       </c>
-      <c r="M2" s="40" t="s">
+      <c r="M2" s="33" t="s">
         <v>13</v>
       </c>
-      <c r="N2" s="40" t="s">
+      <c r="N2" s="33" t="s">
         <v>14</v>
       </c>
-      <c r="O2" s="40" t="s">
+      <c r="O2" s="33" t="s">
         <v>15</v>
       </c>
-      <c r="P2" s="40" t="s">
+      <c r="P2" s="33" t="s">
         <v>16</v>
       </c>
-      <c r="Q2" s="40" t="s">
+      <c r="Q2" s="33" t="s">
         <v>17</v>
       </c>
-      <c r="R2" s="40" t="s">
+      <c r="R2" s="33" t="s">
         <v>18</v>
       </c>
-      <c r="S2" s="40" t="s">
+      <c r="S2" s="33" t="s">
         <v>19</v>
       </c>
-      <c r="T2" s="40" t="s">
+      <c r="T2" s="33" t="s">
         <v>20</v>
       </c>
-      <c r="U2" s="40" t="s">
+      <c r="U2" s="33" t="s">
         <v>21</v>
       </c>
-      <c r="V2" s="40" t="s">
+      <c r="V2" s="33" t="s">
         <v>22</v>
       </c>
-      <c r="W2" s="40" t="s">
+      <c r="W2" s="33" t="s">
         <v>23</v>
       </c>
-      <c r="X2" s="40" t="s">
+      <c r="X2" s="33" t="s">
         <v>24</v>
       </c>
-      <c r="Y2" s="40" t="s">
+      <c r="Y2" s="33" t="s">
         <v>25</v>
       </c>
-      <c r="Z2" s="40" t="s">
+      <c r="Z2" s="33" t="s">
         <v>26</v>
       </c>
-      <c r="AA2" s="40" t="s">
+      <c r="AA2" s="33" t="s">
         <v>27</v>
       </c>
-      <c r="AB2" s="40" t="s">
+      <c r="AB2" s="33" t="s">
         <v>28</v>
       </c>
-      <c r="AC2" s="41" t="s">
+      <c r="AC2" s="34" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="3" spans="1:29" ht="13.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="42"/>
-      <c r="B3" s="43"/>
-      <c r="C3" s="44" t="s">
+    <row r="3" spans="1:29" ht="14" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="35"/>
+      <c r="B3" s="36"/>
+      <c r="C3" s="57" t="s">
         <v>30</v>
       </c>
-      <c r="D3" s="45"/>
-      <c r="E3" s="45"/>
-      <c r="F3" s="45"/>
-      <c r="G3" s="45"/>
-      <c r="H3" s="45"/>
-      <c r="I3" s="45"/>
-      <c r="J3" s="45"/>
-      <c r="K3" s="45"/>
-      <c r="L3" s="45"/>
-      <c r="M3" s="45"/>
-      <c r="N3" s="44" t="s">
+      <c r="D3" s="58"/>
+      <c r="E3" s="58"/>
+      <c r="F3" s="58"/>
+      <c r="G3" s="58"/>
+      <c r="H3" s="58"/>
+      <c r="I3" s="58"/>
+      <c r="J3" s="58"/>
+      <c r="K3" s="58"/>
+      <c r="L3" s="58"/>
+      <c r="M3" s="58"/>
+      <c r="N3" s="57" t="s">
         <v>31</v>
       </c>
-      <c r="O3" s="45"/>
-      <c r="P3" s="45"/>
-      <c r="Q3" s="45"/>
-      <c r="R3" s="45"/>
-      <c r="S3" s="45"/>
-      <c r="T3" s="45"/>
-      <c r="U3" s="45"/>
-      <c r="V3" s="45"/>
-      <c r="W3" s="45"/>
-      <c r="X3" s="45"/>
-      <c r="Y3" s="45"/>
-      <c r="Z3" s="45"/>
-      <c r="AA3" s="45"/>
-      <c r="AB3" s="45"/>
-      <c r="AC3" s="46"/>
+      <c r="O3" s="58"/>
+      <c r="P3" s="58"/>
+      <c r="Q3" s="58"/>
+      <c r="R3" s="58"/>
+      <c r="S3" s="58"/>
+      <c r="T3" s="58"/>
+      <c r="U3" s="58"/>
+      <c r="V3" s="58"/>
+      <c r="W3" s="58"/>
+      <c r="X3" s="58"/>
+      <c r="Y3" s="58"/>
+      <c r="Z3" s="58"/>
+      <c r="AA3" s="58"/>
+      <c r="AB3" s="58"/>
+      <c r="AC3" s="67"/>
     </row>
     <row r="4" spans="1:29" ht="18" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="47" t="s">
+      <c r="A4" s="64" t="s">
         <v>32</v>
       </c>
-      <c r="B4" s="32"/>
-      <c r="C4" s="32"/>
-      <c r="D4" s="32"/>
-      <c r="E4" s="32"/>
-      <c r="F4" s="32"/>
-      <c r="G4" s="32"/>
-      <c r="H4" s="32"/>
-      <c r="I4" s="32"/>
-      <c r="J4" s="32"/>
-      <c r="K4" s="32"/>
-      <c r="L4" s="32"/>
-      <c r="M4" s="32"/>
-      <c r="N4" s="32"/>
-      <c r="O4" s="32"/>
-      <c r="P4" s="32"/>
-      <c r="Q4" s="32"/>
-      <c r="R4" s="32"/>
-      <c r="S4" s="32"/>
-      <c r="T4" s="32"/>
-      <c r="U4" s="32"/>
-      <c r="V4" s="32"/>
-      <c r="W4" s="32"/>
-      <c r="X4" s="32"/>
-      <c r="Y4" s="32"/>
-      <c r="Z4" s="32"/>
-      <c r="AA4" s="32"/>
-      <c r="AB4" s="32"/>
-      <c r="AC4" s="48"/>
+      <c r="B4" s="65"/>
+      <c r="C4" s="65"/>
+      <c r="D4" s="65"/>
+      <c r="E4" s="65"/>
+      <c r="F4" s="65"/>
+      <c r="G4" s="65"/>
+      <c r="H4" s="65"/>
+      <c r="I4" s="65"/>
+      <c r="J4" s="65"/>
+      <c r="K4" s="65"/>
+      <c r="L4" s="65"/>
+      <c r="M4" s="65"/>
+      <c r="N4" s="65"/>
+      <c r="O4" s="65"/>
+      <c r="P4" s="65"/>
+      <c r="Q4" s="65"/>
+      <c r="R4" s="65"/>
+      <c r="S4" s="65"/>
+      <c r="T4" s="65"/>
+      <c r="U4" s="65"/>
+      <c r="V4" s="65"/>
+      <c r="W4" s="65"/>
+      <c r="X4" s="65"/>
+      <c r="Y4" s="65"/>
+      <c r="Z4" s="65"/>
+      <c r="AA4" s="65"/>
+      <c r="AB4" s="65"/>
+      <c r="AC4" s="66"/>
     </row>
     <row r="5" spans="1:29" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="49" t="s">
+      <c r="A5" s="37" t="s">
         <v>61</v>
       </c>
-      <c r="B5" s="28" t="s">
+      <c r="B5" s="25" t="s">
         <v>33</v>
       </c>
       <c r="C5" s="1"/>
@@ -1546,13 +1571,13 @@
       <c r="Z5" s="2"/>
       <c r="AA5" s="2"/>
       <c r="AB5" s="2"/>
-      <c r="AC5" s="50"/>
+      <c r="AC5" s="38"/>
     </row>
     <row r="6" spans="1:29" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="51" t="s">
+      <c r="A6" s="39" t="s">
         <v>68</v>
       </c>
-      <c r="B6" s="27" t="s">
+      <c r="B6" s="24" t="s">
         <v>34</v>
       </c>
       <c r="C6" s="1"/>
@@ -1581,54 +1606,54 @@
       <c r="Z6" s="4"/>
       <c r="AA6" s="4"/>
       <c r="AB6" s="4"/>
-      <c r="AC6" s="50"/>
+      <c r="AC6" s="38"/>
     </row>
     <row r="7" spans="1:29" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="52" t="s">
+      <c r="A7" s="62" t="s">
         <v>35</v>
       </c>
-      <c r="B7" s="18"/>
-      <c r="C7" s="11"/>
-      <c r="D7" s="11"/>
-      <c r="E7" s="11"/>
-      <c r="F7" s="11"/>
-      <c r="G7" s="11"/>
-      <c r="H7" s="11"/>
-      <c r="I7" s="11"/>
-      <c r="J7" s="11"/>
-      <c r="K7" s="11"/>
-      <c r="L7" s="11"/>
-      <c r="M7" s="11"/>
-      <c r="N7" s="11"/>
-      <c r="O7" s="11"/>
-      <c r="P7" s="11"/>
-      <c r="Q7" s="11"/>
-      <c r="R7" s="11"/>
-      <c r="S7" s="11"/>
-      <c r="T7" s="11"/>
-      <c r="U7" s="11"/>
-      <c r="V7" s="11"/>
-      <c r="W7" s="11"/>
-      <c r="X7" s="11"/>
-      <c r="Y7" s="11"/>
-      <c r="Z7" s="11"/>
-      <c r="AA7" s="11"/>
-      <c r="AB7" s="11"/>
+      <c r="B7" s="63"/>
+      <c r="C7" s="52"/>
+      <c r="D7" s="52"/>
+      <c r="E7" s="52"/>
+      <c r="F7" s="52"/>
+      <c r="G7" s="52"/>
+      <c r="H7" s="52"/>
+      <c r="I7" s="52"/>
+      <c r="J7" s="52"/>
+      <c r="K7" s="52"/>
+      <c r="L7" s="52"/>
+      <c r="M7" s="52"/>
+      <c r="N7" s="52"/>
+      <c r="O7" s="52"/>
+      <c r="P7" s="52"/>
+      <c r="Q7" s="52"/>
+      <c r="R7" s="52"/>
+      <c r="S7" s="52"/>
+      <c r="T7" s="52"/>
+      <c r="U7" s="52"/>
+      <c r="V7" s="52"/>
+      <c r="W7" s="52"/>
+      <c r="X7" s="52"/>
+      <c r="Y7" s="52"/>
+      <c r="Z7" s="52"/>
+      <c r="AA7" s="52"/>
+      <c r="AB7" s="52"/>
       <c r="AC7" s="53"/>
     </row>
     <row r="8" spans="1:29" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="54" t="s">
+      <c r="A8" s="40" t="s">
         <v>80</v>
       </c>
-      <c r="B8" s="22" t="s">
+      <c r="B8" s="19" t="s">
         <v>39</v>
       </c>
-      <c r="C8" s="15"/>
+      <c r="C8" s="13"/>
       <c r="D8" s="5"/>
       <c r="E8" s="5"/>
       <c r="F8" s="2"/>
       <c r="G8" s="2"/>
-      <c r="H8" s="19"/>
+      <c r="H8" s="16"/>
       <c r="I8" s="3"/>
       <c r="J8" s="2"/>
       <c r="K8" s="2"/>
@@ -1649,16 +1674,16 @@
       <c r="Z8" s="2"/>
       <c r="AA8" s="2"/>
       <c r="AB8" s="2"/>
-      <c r="AC8" s="50"/>
+      <c r="AC8" s="38"/>
     </row>
     <row r="9" spans="1:29" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="55" t="s">
+      <c r="A9" s="41" t="s">
         <v>112</v>
       </c>
-      <c r="B9" s="23" t="s">
+      <c r="B9" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="C9" s="15"/>
+      <c r="C9" s="13"/>
       <c r="D9" s="5"/>
       <c r="E9" s="5"/>
       <c r="F9" s="4"/>
@@ -1684,16 +1709,16 @@
       <c r="Z9" s="4"/>
       <c r="AA9" s="4"/>
       <c r="AB9" s="4"/>
-      <c r="AC9" s="50"/>
+      <c r="AC9" s="38"/>
     </row>
     <row r="10" spans="1:29" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="54" t="s">
+      <c r="A10" s="40" t="s">
         <v>69</v>
       </c>
-      <c r="B10" s="24" t="s">
+      <c r="B10" s="21" t="s">
         <v>40</v>
       </c>
-      <c r="C10" s="15"/>
+      <c r="C10" s="13"/>
       <c r="D10" s="5"/>
       <c r="E10" s="5"/>
       <c r="F10" s="5"/>
@@ -1701,8 +1726,8 @@
       <c r="H10" s="3"/>
       <c r="I10" s="3"/>
       <c r="J10" s="2"/>
-      <c r="K10" s="20"/>
-      <c r="L10" s="21"/>
+      <c r="K10" s="17"/>
+      <c r="L10" s="18"/>
       <c r="M10" s="2"/>
       <c r="N10" s="2"/>
       <c r="O10" s="3"/>
@@ -1719,16 +1744,16 @@
       <c r="Z10" s="2"/>
       <c r="AA10" s="2"/>
       <c r="AB10" s="2"/>
-      <c r="AC10" s="50"/>
+      <c r="AC10" s="38"/>
     </row>
     <row r="11" spans="1:29" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="55" t="s">
+      <c r="A11" s="41" t="s">
         <v>70</v>
       </c>
-      <c r="B11" s="23" t="s">
+      <c r="B11" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="C11" s="17"/>
+      <c r="C11" s="15"/>
       <c r="D11" s="5"/>
       <c r="E11" s="5"/>
       <c r="F11" s="5"/>
@@ -1754,16 +1779,16 @@
       <c r="Z11" s="4"/>
       <c r="AA11" s="4"/>
       <c r="AB11" s="4"/>
-      <c r="AC11" s="50"/>
+      <c r="AC11" s="38"/>
     </row>
     <row r="12" spans="1:29" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="54" t="s">
+      <c r="A12" s="40" t="s">
         <v>71</v>
       </c>
-      <c r="B12" s="25" t="s">
+      <c r="B12" s="22" t="s">
         <v>36</v>
       </c>
-      <c r="C12" s="15"/>
+      <c r="C12" s="13"/>
       <c r="D12" s="5"/>
       <c r="E12" s="5"/>
       <c r="F12" s="2"/>
@@ -1789,16 +1814,16 @@
       <c r="Z12" s="2"/>
       <c r="AA12" s="2"/>
       <c r="AB12" s="2"/>
-      <c r="AC12" s="50"/>
+      <c r="AC12" s="38"/>
     </row>
     <row r="13" spans="1:29" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="55" t="s">
+      <c r="A13" s="41" t="s">
         <v>37</v>
       </c>
-      <c r="B13" s="26" t="s">
+      <c r="B13" s="23" t="s">
         <v>36</v>
       </c>
-      <c r="C13" s="17"/>
+      <c r="C13" s="15"/>
       <c r="D13" s="4"/>
       <c r="E13" s="5"/>
       <c r="F13" s="5"/>
@@ -1824,16 +1849,16 @@
       <c r="Z13" s="4"/>
       <c r="AA13" s="4"/>
       <c r="AB13" s="4"/>
-      <c r="AC13" s="50"/>
+      <c r="AC13" s="38"/>
     </row>
     <row r="14" spans="1:29" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="54" t="s">
+      <c r="A14" s="40" t="s">
         <v>72</v>
       </c>
-      <c r="B14" s="25" t="s">
+      <c r="B14" s="22" t="s">
         <v>36</v>
       </c>
-      <c r="C14" s="16"/>
+      <c r="C14" s="14"/>
       <c r="D14" s="2"/>
       <c r="E14" s="5"/>
       <c r="F14" s="5"/>
@@ -1859,16 +1884,16 @@
       <c r="Z14" s="2"/>
       <c r="AA14" s="2"/>
       <c r="AB14" s="2"/>
-      <c r="AC14" s="50"/>
+      <c r="AC14" s="38"/>
     </row>
     <row r="15" spans="1:29" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="55" t="s">
+      <c r="A15" s="41" t="s">
         <v>73</v>
       </c>
-      <c r="B15" s="27" t="s">
+      <c r="B15" s="24" t="s">
         <v>34</v>
       </c>
-      <c r="C15" s="17"/>
+      <c r="C15" s="15"/>
       <c r="D15" s="5"/>
       <c r="E15" s="5"/>
       <c r="F15" s="4"/>
@@ -1894,16 +1919,16 @@
       <c r="Z15" s="4"/>
       <c r="AA15" s="4"/>
       <c r="AB15" s="4"/>
-      <c r="AC15" s="50"/>
+      <c r="AC15" s="38"/>
     </row>
     <row r="16" spans="1:29" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="54" t="s">
+      <c r="A16" s="40" t="s">
         <v>74</v>
       </c>
-      <c r="B16" s="28" t="s">
+      <c r="B16" s="25" t="s">
         <v>33</v>
       </c>
-      <c r="C16" s="16"/>
+      <c r="C16" s="14"/>
       <c r="D16" s="5"/>
       <c r="E16" s="5"/>
       <c r="F16" s="5"/>
@@ -1929,16 +1954,16 @@
       <c r="Z16" s="2"/>
       <c r="AA16" s="2"/>
       <c r="AB16" s="2"/>
-      <c r="AC16" s="50"/>
+      <c r="AC16" s="38"/>
     </row>
     <row r="17" spans="1:30" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="55" t="s">
+      <c r="A17" s="41" t="s">
         <v>75</v>
       </c>
-      <c r="B17" s="23" t="s">
+      <c r="B17" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="C17" s="17"/>
+      <c r="C17" s="15"/>
       <c r="D17" s="4"/>
       <c r="E17" s="5"/>
       <c r="F17" s="5"/>
@@ -1964,16 +1989,16 @@
       <c r="Z17" s="4"/>
       <c r="AA17" s="4"/>
       <c r="AB17" s="4"/>
-      <c r="AC17" s="50"/>
+      <c r="AC17" s="38"/>
     </row>
     <row r="18" spans="1:30" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="54" t="s">
+      <c r="A18" s="40" t="s">
         <v>77</v>
       </c>
-      <c r="B18" s="25" t="s">
+      <c r="B18" s="22" t="s">
         <v>36</v>
       </c>
-      <c r="C18" s="16"/>
+      <c r="C18" s="14"/>
       <c r="D18" s="2"/>
       <c r="E18" s="5"/>
       <c r="F18" s="5"/>
@@ -1999,16 +2024,16 @@
       <c r="Z18" s="2"/>
       <c r="AA18" s="2"/>
       <c r="AB18" s="2"/>
-      <c r="AC18" s="50"/>
+      <c r="AC18" s="38"/>
     </row>
     <row r="19" spans="1:30" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="55" t="s">
+      <c r="A19" s="41" t="s">
         <v>76</v>
       </c>
-      <c r="B19" s="23" t="s">
+      <c r="B19" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="C19" s="17"/>
+      <c r="C19" s="15"/>
       <c r="D19" s="4"/>
       <c r="E19" s="5"/>
       <c r="F19" s="5"/>
@@ -2034,16 +2059,16 @@
       <c r="Z19" s="4"/>
       <c r="AA19" s="4"/>
       <c r="AB19" s="4"/>
-      <c r="AC19" s="50"/>
+      <c r="AC19" s="38"/>
     </row>
     <row r="20" spans="1:30" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="54" t="s">
+      <c r="A20" s="40" t="s">
         <v>78</v>
       </c>
-      <c r="B20" s="29" t="s">
+      <c r="B20" s="26" t="s">
         <v>34</v>
       </c>
-      <c r="C20" s="16"/>
+      <c r="C20" s="14"/>
       <c r="D20" s="2"/>
       <c r="E20" s="2"/>
       <c r="F20" s="2"/>
@@ -2069,16 +2094,16 @@
       <c r="Z20" s="2"/>
       <c r="AA20" s="2"/>
       <c r="AB20" s="2"/>
-      <c r="AC20" s="50"/>
+      <c r="AC20" s="38"/>
     </row>
     <row r="21" spans="1:30" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="55" t="s">
+      <c r="A21" s="41" t="s">
         <v>79</v>
       </c>
-      <c r="B21" s="27" t="s">
+      <c r="B21" s="24" t="s">
         <v>34</v>
       </c>
-      <c r="C21" s="17"/>
+      <c r="C21" s="15"/>
       <c r="D21" s="4"/>
       <c r="E21" s="4"/>
       <c r="F21" s="4"/>
@@ -2104,46 +2129,46 @@
       <c r="Z21" s="4"/>
       <c r="AA21" s="4"/>
       <c r="AB21" s="4"/>
-      <c r="AC21" s="50"/>
+      <c r="AC21" s="38"/>
     </row>
     <row r="22" spans="1:30" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="56" t="s">
+      <c r="A22" s="51" t="s">
         <v>38</v>
       </c>
-      <c r="B22" s="11"/>
-      <c r="C22" s="11"/>
-      <c r="D22" s="11"/>
-      <c r="E22" s="11"/>
-      <c r="F22" s="11"/>
-      <c r="G22" s="11"/>
-      <c r="H22" s="11"/>
-      <c r="I22" s="11"/>
-      <c r="J22" s="11"/>
-      <c r="K22" s="11"/>
-      <c r="L22" s="11"/>
-      <c r="M22" s="11"/>
-      <c r="N22" s="11"/>
-      <c r="O22" s="11"/>
-      <c r="P22" s="11"/>
-      <c r="Q22" s="11"/>
-      <c r="R22" s="11"/>
-      <c r="S22" s="11"/>
-      <c r="T22" s="11"/>
-      <c r="U22" s="11"/>
-      <c r="V22" s="11"/>
-      <c r="W22" s="11"/>
-      <c r="X22" s="11"/>
-      <c r="Y22" s="11"/>
-      <c r="Z22" s="11"/>
-      <c r="AA22" s="11"/>
-      <c r="AB22" s="11"/>
+      <c r="B22" s="52"/>
+      <c r="C22" s="52"/>
+      <c r="D22" s="52"/>
+      <c r="E22" s="52"/>
+      <c r="F22" s="52"/>
+      <c r="G22" s="52"/>
+      <c r="H22" s="52"/>
+      <c r="I22" s="52"/>
+      <c r="J22" s="52"/>
+      <c r="K22" s="52"/>
+      <c r="L22" s="52"/>
+      <c r="M22" s="52"/>
+      <c r="N22" s="52"/>
+      <c r="O22" s="52"/>
+      <c r="P22" s="52"/>
+      <c r="Q22" s="52"/>
+      <c r="R22" s="52"/>
+      <c r="S22" s="52"/>
+      <c r="T22" s="52"/>
+      <c r="U22" s="52"/>
+      <c r="V22" s="52"/>
+      <c r="W22" s="52"/>
+      <c r="X22" s="52"/>
+      <c r="Y22" s="52"/>
+      <c r="Z22" s="52"/>
+      <c r="AA22" s="52"/>
+      <c r="AB22" s="52"/>
       <c r="AC22" s="53"/>
     </row>
     <row r="23" spans="1:30" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="54" t="s">
+      <c r="A23" s="40" t="s">
         <v>81</v>
       </c>
-      <c r="B23" s="22" t="s">
+      <c r="B23" s="19" t="s">
         <v>39</v>
       </c>
       <c r="C23" s="2"/>
@@ -2172,13 +2197,13 @@
       <c r="Z23" s="2"/>
       <c r="AA23" s="2"/>
       <c r="AB23" s="2"/>
-      <c r="AC23" s="50"/>
+      <c r="AC23" s="38"/>
     </row>
     <row r="24" spans="1:30" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="55" t="s">
+      <c r="A24" s="41" t="s">
         <v>82</v>
       </c>
-      <c r="B24" s="30" t="s">
+      <c r="B24" s="27" t="s">
         <v>40</v>
       </c>
       <c r="C24" s="4"/>
@@ -2209,13 +2234,13 @@
       <c r="Z24" s="4"/>
       <c r="AA24" s="4"/>
       <c r="AB24" s="4"/>
-      <c r="AC24" s="50"/>
+      <c r="AC24" s="38"/>
     </row>
     <row r="25" spans="1:30" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="54" t="s">
+      <c r="A25" s="40" t="s">
         <v>83</v>
       </c>
-      <c r="B25" s="25" t="s">
+      <c r="B25" s="22" t="s">
         <v>36</v>
       </c>
       <c r="C25" s="2"/>
@@ -2244,13 +2269,13 @@
       <c r="Z25" s="2"/>
       <c r="AA25" s="2"/>
       <c r="AB25" s="2"/>
-      <c r="AC25" s="50"/>
+      <c r="AC25" s="38"/>
     </row>
     <row r="26" spans="1:30" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="55" t="s">
+      <c r="A26" s="41" t="s">
         <v>84</v>
       </c>
-      <c r="B26" s="31" t="s">
+      <c r="B26" s="28" t="s">
         <v>39</v>
       </c>
       <c r="C26" s="4"/>
@@ -2279,13 +2304,13 @@
       <c r="Z26" s="4"/>
       <c r="AA26" s="4"/>
       <c r="AB26" s="4"/>
-      <c r="AC26" s="50"/>
+      <c r="AC26" s="38"/>
     </row>
     <row r="27" spans="1:30" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="54" t="s">
+      <c r="A27" s="40" t="s">
         <v>85</v>
       </c>
-      <c r="B27" s="25" t="s">
+      <c r="B27" s="22" t="s">
         <v>36</v>
       </c>
       <c r="C27" s="2"/>
@@ -2314,13 +2339,13 @@
       <c r="Z27" s="2"/>
       <c r="AA27" s="2"/>
       <c r="AB27" s="2"/>
-      <c r="AC27" s="50"/>
+      <c r="AC27" s="38"/>
     </row>
     <row r="28" spans="1:30" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A28" s="55" t="s">
+      <c r="A28" s="41" t="s">
         <v>86</v>
       </c>
-      <c r="B28" s="26" t="s">
+      <c r="B28" s="23" t="s">
         <v>36</v>
       </c>
       <c r="C28" s="4"/>
@@ -2349,14 +2374,14 @@
       <c r="Z28" s="4"/>
       <c r="AA28" s="4"/>
       <c r="AB28" s="4"/>
-      <c r="AC28" s="50"/>
-      <c r="AD28" s="33"/>
+      <c r="AC28" s="38"/>
+      <c r="AD28" s="29"/>
     </row>
     <row r="29" spans="1:30" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="54" t="s">
+      <c r="A29" s="40" t="s">
         <v>87</v>
       </c>
-      <c r="B29" s="22" t="s">
+      <c r="B29" s="19" t="s">
         <v>39</v>
       </c>
       <c r="C29" s="2"/>
@@ -2385,13 +2410,13 @@
       <c r="Z29" s="2"/>
       <c r="AA29" s="2"/>
       <c r="AB29" s="2"/>
-      <c r="AC29" s="50"/>
+      <c r="AC29" s="38"/>
     </row>
     <row r="30" spans="1:30" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="55" t="s">
+      <c r="A30" s="41" t="s">
         <v>88</v>
       </c>
-      <c r="B30" s="31" t="s">
+      <c r="B30" s="28" t="s">
         <v>39</v>
       </c>
       <c r="C30" s="4"/>
@@ -2420,13 +2445,13 @@
       <c r="Z30" s="4"/>
       <c r="AA30" s="4"/>
       <c r="AB30" s="4"/>
-      <c r="AC30" s="50"/>
+      <c r="AC30" s="38"/>
     </row>
     <row r="31" spans="1:30" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="54" t="s">
+      <c r="A31" s="40" t="s">
         <v>89</v>
       </c>
-      <c r="B31" s="22" t="s">
+      <c r="B31" s="19" t="s">
         <v>39</v>
       </c>
       <c r="C31" s="2"/>
@@ -2455,13 +2480,13 @@
       <c r="Z31" s="2"/>
       <c r="AA31" s="2"/>
       <c r="AB31" s="2"/>
-      <c r="AC31" s="50"/>
+      <c r="AC31" s="38"/>
     </row>
     <row r="32" spans="1:30" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="55" t="s">
+      <c r="A32" s="41" t="s">
         <v>113</v>
       </c>
-      <c r="B32" s="30" t="s">
+      <c r="B32" s="27" t="s">
         <v>40</v>
       </c>
       <c r="C32" s="4"/>
@@ -2490,13 +2515,13 @@
       <c r="Z32" s="4"/>
       <c r="AA32" s="4"/>
       <c r="AB32" s="4"/>
-      <c r="AC32" s="50"/>
+      <c r="AC32" s="38"/>
     </row>
     <row r="33" spans="1:29" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="54" t="s">
+      <c r="A33" s="40" t="s">
         <v>114</v>
       </c>
-      <c r="B33" s="24" t="s">
+      <c r="B33" s="21" t="s">
         <v>40</v>
       </c>
       <c r="C33" s="2"/>
@@ -2525,13 +2550,13 @@
       <c r="Z33" s="2"/>
       <c r="AA33" s="2"/>
       <c r="AB33" s="2"/>
-      <c r="AC33" s="50"/>
+      <c r="AC33" s="38"/>
     </row>
     <row r="34" spans="1:29" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="55" t="s">
+      <c r="A34" s="41" t="s">
         <v>90</v>
       </c>
-      <c r="B34" s="23" t="s">
+      <c r="B34" s="20" t="s">
         <v>33</v>
       </c>
       <c r="C34" s="4"/>
@@ -2560,13 +2585,13 @@
       <c r="Z34" s="4"/>
       <c r="AA34" s="4"/>
       <c r="AB34" s="4"/>
-      <c r="AC34" s="50"/>
+      <c r="AC34" s="38"/>
     </row>
     <row r="35" spans="1:29" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="54" t="s">
+      <c r="A35" s="40" t="s">
         <v>91</v>
       </c>
-      <c r="B35" s="28" t="s">
+      <c r="B35" s="25" t="s">
         <v>33</v>
       </c>
       <c r="C35" s="2"/>
@@ -2595,13 +2620,13 @@
       <c r="Z35" s="2"/>
       <c r="AA35" s="2"/>
       <c r="AB35" s="2"/>
-      <c r="AC35" s="50"/>
+      <c r="AC35" s="38"/>
     </row>
     <row r="36" spans="1:29" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="55" t="s">
+      <c r="A36" s="41" t="s">
         <v>62</v>
       </c>
-      <c r="B36" s="23" t="s">
+      <c r="B36" s="20" t="s">
         <v>33</v>
       </c>
       <c r="C36" s="4"/>
@@ -2630,46 +2655,46 @@
       <c r="Z36" s="4"/>
       <c r="AA36" s="4"/>
       <c r="AB36" s="4"/>
-      <c r="AC36" s="50"/>
+      <c r="AC36" s="38"/>
     </row>
     <row r="37" spans="1:29" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="56" t="s">
+      <c r="A37" s="51" t="s">
         <v>41</v>
       </c>
-      <c r="B37" s="11"/>
-      <c r="C37" s="11"/>
-      <c r="D37" s="11"/>
-      <c r="E37" s="11"/>
-      <c r="F37" s="11"/>
-      <c r="G37" s="11"/>
-      <c r="H37" s="11"/>
-      <c r="I37" s="11"/>
-      <c r="J37" s="11"/>
-      <c r="K37" s="11"/>
-      <c r="L37" s="11"/>
-      <c r="M37" s="11"/>
-      <c r="N37" s="11"/>
-      <c r="O37" s="11"/>
-      <c r="P37" s="11"/>
-      <c r="Q37" s="11"/>
-      <c r="R37" s="11"/>
-      <c r="S37" s="11"/>
-      <c r="T37" s="11"/>
-      <c r="U37" s="11"/>
-      <c r="V37" s="11"/>
-      <c r="W37" s="11"/>
-      <c r="X37" s="11"/>
-      <c r="Y37" s="11"/>
-      <c r="Z37" s="11"/>
-      <c r="AA37" s="11"/>
-      <c r="AB37" s="11"/>
+      <c r="B37" s="52"/>
+      <c r="C37" s="52"/>
+      <c r="D37" s="52"/>
+      <c r="E37" s="52"/>
+      <c r="F37" s="52"/>
+      <c r="G37" s="52"/>
+      <c r="H37" s="52"/>
+      <c r="I37" s="52"/>
+      <c r="J37" s="52"/>
+      <c r="K37" s="52"/>
+      <c r="L37" s="52"/>
+      <c r="M37" s="52"/>
+      <c r="N37" s="52"/>
+      <c r="O37" s="52"/>
+      <c r="P37" s="52"/>
+      <c r="Q37" s="52"/>
+      <c r="R37" s="52"/>
+      <c r="S37" s="52"/>
+      <c r="T37" s="52"/>
+      <c r="U37" s="52"/>
+      <c r="V37" s="52"/>
+      <c r="W37" s="52"/>
+      <c r="X37" s="52"/>
+      <c r="Y37" s="52"/>
+      <c r="Z37" s="52"/>
+      <c r="AA37" s="52"/>
+      <c r="AB37" s="52"/>
       <c r="AC37" s="53"/>
     </row>
     <row r="38" spans="1:29" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="54" t="s">
+      <c r="A38" s="40" t="s">
         <v>92</v>
       </c>
-      <c r="B38" s="22" t="s">
+      <c r="B38" s="19" t="s">
         <v>39</v>
       </c>
       <c r="C38" s="2"/>
@@ -2698,13 +2723,13 @@
       <c r="Z38" s="2"/>
       <c r="AA38" s="2"/>
       <c r="AB38" s="2"/>
-      <c r="AC38" s="50"/>
+      <c r="AC38" s="38"/>
     </row>
     <row r="39" spans="1:29" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="55" t="s">
+      <c r="A39" s="41" t="s">
         <v>93</v>
       </c>
-      <c r="B39" s="31" t="s">
+      <c r="B39" s="28" t="s">
         <v>39</v>
       </c>
       <c r="C39" s="4"/>
@@ -2733,13 +2758,13 @@
       <c r="Z39" s="4"/>
       <c r="AA39" s="4"/>
       <c r="AB39" s="4"/>
-      <c r="AC39" s="50"/>
+      <c r="AC39" s="38"/>
     </row>
     <row r="40" spans="1:29" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A40" s="54" t="s">
+      <c r="A40" s="40" t="s">
         <v>94</v>
       </c>
-      <c r="B40" s="22" t="s">
+      <c r="B40" s="19" t="s">
         <v>39</v>
       </c>
       <c r="C40" s="2"/>
@@ -2768,13 +2793,13 @@
       <c r="Z40" s="2"/>
       <c r="AA40" s="2"/>
       <c r="AB40" s="2"/>
-      <c r="AC40" s="50"/>
+      <c r="AC40" s="38"/>
     </row>
     <row r="41" spans="1:29" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="55" t="s">
+      <c r="A41" s="41" t="s">
         <v>42</v>
       </c>
-      <c r="B41" s="31" t="s">
+      <c r="B41" s="28" t="s">
         <v>39</v>
       </c>
       <c r="C41" s="4"/>
@@ -2803,13 +2828,13 @@
       <c r="Z41" s="4"/>
       <c r="AA41" s="4"/>
       <c r="AB41" s="4"/>
-      <c r="AC41" s="50"/>
+      <c r="AC41" s="38"/>
     </row>
     <row r="42" spans="1:29" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="54" t="s">
+      <c r="A42" s="40" t="s">
         <v>95</v>
       </c>
-      <c r="B42" s="22" t="s">
+      <c r="B42" s="19" t="s">
         <v>39</v>
       </c>
       <c r="C42" s="2"/>
@@ -2838,13 +2863,13 @@
       <c r="Z42" s="2"/>
       <c r="AA42" s="2"/>
       <c r="AB42" s="2"/>
-      <c r="AC42" s="50"/>
+      <c r="AC42" s="38"/>
     </row>
     <row r="43" spans="1:29" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="55" t="s">
+      <c r="A43" s="41" t="s">
         <v>43</v>
       </c>
-      <c r="B43" s="30" t="s">
+      <c r="B43" s="27" t="s">
         <v>40</v>
       </c>
       <c r="C43" s="4"/>
@@ -2873,13 +2898,13 @@
       <c r="Z43" s="4"/>
       <c r="AA43" s="4"/>
       <c r="AB43" s="4"/>
-      <c r="AC43" s="50"/>
+      <c r="AC43" s="38"/>
     </row>
     <row r="44" spans="1:29" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="54" t="s">
+      <c r="A44" s="40" t="s">
         <v>44</v>
       </c>
-      <c r="B44" s="24" t="s">
+      <c r="B44" s="21" t="s">
         <v>40</v>
       </c>
       <c r="C44" s="2"/>
@@ -2908,13 +2933,13 @@
       <c r="Z44" s="2"/>
       <c r="AA44" s="2"/>
       <c r="AB44" s="2"/>
-      <c r="AC44" s="50"/>
+      <c r="AC44" s="38"/>
     </row>
     <row r="45" spans="1:29" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="55" t="s">
+      <c r="A45" s="41" t="s">
         <v>96</v>
       </c>
-      <c r="B45" s="23" t="s">
+      <c r="B45" s="20" t="s">
         <v>33</v>
       </c>
       <c r="C45" s="4"/>
@@ -2943,13 +2968,13 @@
       <c r="Z45" s="4"/>
       <c r="AA45" s="4"/>
       <c r="AB45" s="4"/>
-      <c r="AC45" s="50"/>
+      <c r="AC45" s="38"/>
     </row>
     <row r="46" spans="1:29" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="54" t="s">
+      <c r="A46" s="40" t="s">
         <v>63</v>
       </c>
-      <c r="B46" s="28" t="s">
+      <c r="B46" s="25" t="s">
         <v>33</v>
       </c>
       <c r="C46" s="2"/>
@@ -2978,13 +3003,13 @@
       <c r="Z46" s="2"/>
       <c r="AA46" s="2"/>
       <c r="AB46" s="2"/>
-      <c r="AC46" s="57"/>
+      <c r="AC46" s="42"/>
     </row>
     <row r="47" spans="1:29" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="55" t="s">
+      <c r="A47" s="41" t="s">
         <v>64</v>
       </c>
-      <c r="B47" s="23" t="s">
+      <c r="B47" s="20" t="s">
         <v>33</v>
       </c>
       <c r="C47" s="4"/>
@@ -3013,13 +3038,13 @@
       <c r="Z47" s="4"/>
       <c r="AA47" s="4"/>
       <c r="AB47" s="4"/>
-      <c r="AC47" s="57"/>
+      <c r="AC47" s="42"/>
     </row>
     <row r="48" spans="1:29" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="54" t="s">
+      <c r="A48" s="40" t="s">
         <v>97</v>
       </c>
-      <c r="B48" s="28" t="s">
+      <c r="B48" s="25" t="s">
         <v>33</v>
       </c>
       <c r="C48" s="2"/>
@@ -3048,13 +3073,13 @@
       <c r="Z48" s="2"/>
       <c r="AA48" s="2"/>
       <c r="AB48" s="2"/>
-      <c r="AC48" s="57"/>
+      <c r="AC48" s="42"/>
     </row>
     <row r="49" spans="1:29" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="55" t="s">
+      <c r="A49" s="41" t="s">
         <v>65</v>
       </c>
-      <c r="B49" s="23" t="s">
+      <c r="B49" s="20" t="s">
         <v>33</v>
       </c>
       <c r="C49" s="4"/>
@@ -3062,8 +3087,8 @@
       <c r="E49" s="4"/>
       <c r="F49" s="4"/>
       <c r="G49" s="4"/>
-      <c r="H49" s="12"/>
-      <c r="I49" s="12"/>
+      <c r="H49" s="11"/>
+      <c r="I49" s="11"/>
       <c r="J49" s="4"/>
       <c r="K49" s="4"/>
       <c r="L49" s="4"/>
@@ -3083,13 +3108,13 @@
       <c r="Z49" s="4"/>
       <c r="AA49" s="4"/>
       <c r="AB49" s="4"/>
-      <c r="AC49" s="57"/>
+      <c r="AC49" s="42"/>
     </row>
     <row r="50" spans="1:29" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="54" t="s">
+      <c r="A50" s="40" t="s">
         <v>66</v>
       </c>
-      <c r="B50" s="28" t="s">
+      <c r="B50" s="25" t="s">
         <v>33</v>
       </c>
       <c r="C50" s="2"/>
@@ -3097,8 +3122,8 @@
       <c r="E50" s="2"/>
       <c r="F50" s="2"/>
       <c r="G50" s="2"/>
-      <c r="H50" s="12"/>
-      <c r="I50" s="12"/>
+      <c r="H50" s="11"/>
+      <c r="I50" s="11"/>
       <c r="J50" s="2"/>
       <c r="K50" s="2"/>
       <c r="L50" s="2"/>
@@ -3118,46 +3143,46 @@
       <c r="Z50" s="2"/>
       <c r="AA50" s="2"/>
       <c r="AB50" s="2"/>
-      <c r="AC50" s="57"/>
+      <c r="AC50" s="42"/>
     </row>
     <row r="51" spans="1:29" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="56" t="s">
+      <c r="A51" s="51" t="s">
         <v>45</v>
       </c>
-      <c r="B51" s="11"/>
-      <c r="C51" s="11"/>
-      <c r="D51" s="11"/>
-      <c r="E51" s="11"/>
-      <c r="F51" s="11"/>
-      <c r="G51" s="11"/>
-      <c r="H51" s="11"/>
-      <c r="I51" s="11"/>
-      <c r="J51" s="11"/>
-      <c r="K51" s="11"/>
-      <c r="L51" s="11"/>
-      <c r="M51" s="11"/>
-      <c r="N51" s="11"/>
-      <c r="O51" s="11"/>
-      <c r="P51" s="11"/>
-      <c r="Q51" s="11"/>
-      <c r="R51" s="11"/>
-      <c r="S51" s="11"/>
-      <c r="T51" s="11"/>
-      <c r="U51" s="11"/>
-      <c r="V51" s="11"/>
-      <c r="W51" s="11"/>
-      <c r="X51" s="11"/>
-      <c r="Y51" s="11"/>
-      <c r="Z51" s="11"/>
-      <c r="AA51" s="11"/>
-      <c r="AB51" s="11"/>
+      <c r="B51" s="52"/>
+      <c r="C51" s="52"/>
+      <c r="D51" s="52"/>
+      <c r="E51" s="52"/>
+      <c r="F51" s="52"/>
+      <c r="G51" s="52"/>
+      <c r="H51" s="52"/>
+      <c r="I51" s="52"/>
+      <c r="J51" s="52"/>
+      <c r="K51" s="52"/>
+      <c r="L51" s="52"/>
+      <c r="M51" s="52"/>
+      <c r="N51" s="52"/>
+      <c r="O51" s="52"/>
+      <c r="P51" s="52"/>
+      <c r="Q51" s="52"/>
+      <c r="R51" s="52"/>
+      <c r="S51" s="52"/>
+      <c r="T51" s="52"/>
+      <c r="U51" s="52"/>
+      <c r="V51" s="52"/>
+      <c r="W51" s="52"/>
+      <c r="X51" s="52"/>
+      <c r="Y51" s="52"/>
+      <c r="Z51" s="52"/>
+      <c r="AA51" s="52"/>
+      <c r="AB51" s="52"/>
       <c r="AC51" s="53"/>
     </row>
     <row r="52" spans="1:29" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A52" s="54" t="s">
+      <c r="A52" s="40" t="s">
         <v>98</v>
       </c>
-      <c r="B52" s="22" t="s">
+      <c r="B52" s="19" t="s">
         <v>39</v>
       </c>
       <c r="C52" s="2"/>
@@ -3186,13 +3211,13 @@
       <c r="Z52" s="2"/>
       <c r="AA52" s="2"/>
       <c r="AB52" s="2"/>
-      <c r="AC52" s="50"/>
+      <c r="AC52" s="38"/>
     </row>
     <row r="53" spans="1:29" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A53" s="55" t="s">
+      <c r="A53" s="41" t="s">
         <v>99</v>
       </c>
-      <c r="B53" s="31" t="s">
+      <c r="B53" s="28" t="s">
         <v>39</v>
       </c>
       <c r="C53" s="4"/>
@@ -3221,13 +3246,13 @@
       <c r="Z53" s="4"/>
       <c r="AA53" s="4"/>
       <c r="AB53" s="4"/>
-      <c r="AC53" s="50"/>
+      <c r="AC53" s="38"/>
     </row>
     <row r="54" spans="1:29" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A54" s="58" t="s">
+      <c r="A54" s="43" t="s">
         <v>100</v>
       </c>
-      <c r="B54" s="22" t="s">
+      <c r="B54" s="19" t="s">
         <v>39</v>
       </c>
       <c r="C54" s="2"/>
@@ -3256,13 +3281,13 @@
       <c r="Z54" s="2"/>
       <c r="AA54" s="2"/>
       <c r="AB54" s="2"/>
-      <c r="AC54" s="50"/>
+      <c r="AC54" s="38"/>
     </row>
     <row r="55" spans="1:29" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A55" s="59" t="s">
+      <c r="A55" s="44" t="s">
         <v>101</v>
       </c>
-      <c r="B55" s="31" t="s">
+      <c r="B55" s="28" t="s">
         <v>39</v>
       </c>
       <c r="C55" s="4"/>
@@ -3291,13 +3316,13 @@
       <c r="Z55" s="4"/>
       <c r="AA55" s="4"/>
       <c r="AB55" s="4"/>
-      <c r="AC55" s="50"/>
+      <c r="AC55" s="38"/>
     </row>
     <row r="56" spans="1:29" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A56" s="54" t="s">
+      <c r="A56" s="40" t="s">
         <v>46</v>
       </c>
-      <c r="B56" s="24" t="s">
+      <c r="B56" s="21" t="s">
         <v>40</v>
       </c>
       <c r="C56" s="2"/>
@@ -3326,13 +3351,13 @@
       <c r="Z56" s="2"/>
       <c r="AA56" s="2"/>
       <c r="AB56" s="2"/>
-      <c r="AC56" s="50"/>
+      <c r="AC56" s="38"/>
     </row>
     <row r="57" spans="1:29" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A57" s="55" t="s">
+      <c r="A57" s="41" t="s">
         <v>102</v>
       </c>
-      <c r="B57" s="23" t="s">
+      <c r="B57" s="20" t="s">
         <v>33</v>
       </c>
       <c r="C57" s="4"/>
@@ -3361,13 +3386,13 @@
       <c r="Z57" s="4"/>
       <c r="AA57" s="4"/>
       <c r="AB57" s="4"/>
-      <c r="AC57" s="50"/>
+      <c r="AC57" s="38"/>
     </row>
     <row r="58" spans="1:29" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A58" s="54" t="s">
+      <c r="A58" s="40" t="s">
         <v>103</v>
       </c>
-      <c r="B58" s="28" t="s">
+      <c r="B58" s="25" t="s">
         <v>33</v>
       </c>
       <c r="C58" s="2"/>
@@ -3396,13 +3421,13 @@
       <c r="Z58" s="2"/>
       <c r="AA58" s="2"/>
       <c r="AB58" s="2"/>
-      <c r="AC58" s="50"/>
+      <c r="AC58" s="38"/>
     </row>
     <row r="59" spans="1:29" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A59" s="55" t="s">
+      <c r="A59" s="41" t="s">
         <v>49</v>
       </c>
-      <c r="B59" s="23" t="s">
+      <c r="B59" s="20" t="s">
         <v>33</v>
       </c>
       <c r="C59" s="4"/>
@@ -3431,13 +3456,13 @@
       <c r="Z59" s="8"/>
       <c r="AA59" s="4"/>
       <c r="AB59" s="4"/>
-      <c r="AC59" s="50"/>
+      <c r="AC59" s="38"/>
     </row>
     <row r="60" spans="1:29" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A60" s="54" t="s">
+      <c r="A60" s="40" t="s">
         <v>47</v>
       </c>
-      <c r="B60" s="22" t="s">
+      <c r="B60" s="19" t="s">
         <v>39</v>
       </c>
       <c r="C60" s="2"/>
@@ -3466,13 +3491,13 @@
       <c r="Z60" s="8"/>
       <c r="AA60" s="2"/>
       <c r="AB60" s="2"/>
-      <c r="AC60" s="57"/>
+      <c r="AC60" s="42"/>
     </row>
     <row r="61" spans="1:29" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A61" s="55" t="s">
+      <c r="A61" s="41" t="s">
         <v>104</v>
       </c>
-      <c r="B61" s="23" t="s">
+      <c r="B61" s="20" t="s">
         <v>33</v>
       </c>
       <c r="C61" s="4"/>
@@ -3501,13 +3526,13 @@
       <c r="Z61" s="8"/>
       <c r="AA61" s="4"/>
       <c r="AB61" s="4"/>
-      <c r="AC61" s="50"/>
+      <c r="AC61" s="38"/>
     </row>
     <row r="62" spans="1:29" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A62" s="54" t="s">
+      <c r="A62" s="40" t="s">
         <v>105</v>
       </c>
-      <c r="B62" s="24" t="s">
+      <c r="B62" s="21" t="s">
         <v>40</v>
       </c>
       <c r="C62" s="2"/>
@@ -3515,15 +3540,15 @@
       <c r="E62" s="2"/>
       <c r="F62" s="2"/>
       <c r="G62" s="2"/>
-      <c r="H62" s="12"/>
-      <c r="I62" s="12"/>
+      <c r="H62" s="11"/>
+      <c r="I62" s="11"/>
       <c r="J62" s="2"/>
       <c r="K62" s="2"/>
       <c r="L62" s="2"/>
       <c r="M62" s="2"/>
       <c r="N62" s="2"/>
-      <c r="O62" s="12"/>
-      <c r="P62" s="12"/>
+      <c r="O62" s="11"/>
+      <c r="P62" s="11"/>
       <c r="Q62" s="2"/>
       <c r="R62" s="2"/>
       <c r="S62" s="2"/>
@@ -3536,13 +3561,13 @@
       <c r="Z62" s="8"/>
       <c r="AA62" s="2"/>
       <c r="AB62" s="2"/>
-      <c r="AC62" s="57"/>
+      <c r="AC62" s="42"/>
     </row>
     <row r="63" spans="1:29" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A63" s="55" t="s">
+      <c r="A63" s="41" t="s">
         <v>106</v>
       </c>
-      <c r="B63" s="27" t="s">
+      <c r="B63" s="24" t="s">
         <v>34</v>
       </c>
       <c r="C63" s="4"/>
@@ -3550,15 +3575,15 @@
       <c r="E63" s="4"/>
       <c r="F63" s="4"/>
       <c r="G63" s="4"/>
-      <c r="H63" s="12"/>
-      <c r="I63" s="12"/>
+      <c r="H63" s="11"/>
+      <c r="I63" s="11"/>
       <c r="J63" s="4"/>
       <c r="K63" s="4"/>
       <c r="L63" s="4"/>
       <c r="M63" s="4"/>
       <c r="N63" s="4"/>
-      <c r="O63" s="12"/>
-      <c r="P63" s="12"/>
+      <c r="O63" s="11"/>
+      <c r="P63" s="11"/>
       <c r="Q63" s="4"/>
       <c r="R63" s="4"/>
       <c r="S63" s="4"/>
@@ -3571,46 +3596,46 @@
       <c r="Z63" s="4"/>
       <c r="AA63" s="8"/>
       <c r="AB63" s="4"/>
-      <c r="AC63" s="57"/>
+      <c r="AC63" s="42"/>
     </row>
     <row r="64" spans="1:29" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A64" s="60" t="s">
+      <c r="A64" s="59" t="s">
         <v>48</v>
       </c>
-      <c r="B64" s="13"/>
-      <c r="C64" s="13"/>
-      <c r="D64" s="13"/>
-      <c r="E64" s="13"/>
-      <c r="F64" s="13"/>
-      <c r="G64" s="13"/>
-      <c r="H64" s="13"/>
-      <c r="I64" s="13"/>
-      <c r="J64" s="13"/>
-      <c r="K64" s="13"/>
-      <c r="L64" s="13"/>
-      <c r="M64" s="13"/>
-      <c r="N64" s="13"/>
-      <c r="O64" s="13"/>
-      <c r="P64" s="13"/>
-      <c r="Q64" s="13"/>
-      <c r="R64" s="13"/>
-      <c r="S64" s="13"/>
-      <c r="T64" s="13"/>
-      <c r="U64" s="13"/>
-      <c r="V64" s="13"/>
-      <c r="W64" s="13"/>
-      <c r="X64" s="13"/>
-      <c r="Y64" s="13"/>
-      <c r="Z64" s="13"/>
-      <c r="AA64" s="13"/>
-      <c r="AB64" s="13"/>
+      <c r="B64" s="60"/>
+      <c r="C64" s="60"/>
+      <c r="D64" s="60"/>
+      <c r="E64" s="60"/>
+      <c r="F64" s="60"/>
+      <c r="G64" s="60"/>
+      <c r="H64" s="60"/>
+      <c r="I64" s="60"/>
+      <c r="J64" s="60"/>
+      <c r="K64" s="60"/>
+      <c r="L64" s="60"/>
+      <c r="M64" s="60"/>
+      <c r="N64" s="60"/>
+      <c r="O64" s="60"/>
+      <c r="P64" s="60"/>
+      <c r="Q64" s="60"/>
+      <c r="R64" s="60"/>
+      <c r="S64" s="60"/>
+      <c r="T64" s="60"/>
+      <c r="U64" s="60"/>
+      <c r="V64" s="60"/>
+      <c r="W64" s="60"/>
+      <c r="X64" s="60"/>
+      <c r="Y64" s="60"/>
+      <c r="Z64" s="60"/>
+      <c r="AA64" s="60"/>
+      <c r="AB64" s="60"/>
       <c r="AC64" s="61"/>
     </row>
     <row r="65" spans="1:29" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A65" s="54" t="s">
+      <c r="A65" s="40" t="s">
         <v>107</v>
       </c>
-      <c r="B65" s="28" t="s">
+      <c r="B65" s="25" t="s">
         <v>33</v>
       </c>
       <c r="C65" s="2"/>
@@ -3639,13 +3664,13 @@
       <c r="Z65" s="2"/>
       <c r="AA65" s="1"/>
       <c r="AB65" s="1"/>
-      <c r="AC65" s="50"/>
+      <c r="AC65" s="38"/>
     </row>
     <row r="66" spans="1:29" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A66" s="55" t="s">
+      <c r="A66" s="41" t="s">
         <v>108</v>
       </c>
-      <c r="B66" s="23" t="s">
+      <c r="B66" s="20" t="s">
         <v>33</v>
       </c>
       <c r="C66" s="4"/>
@@ -3674,13 +3699,13 @@
       <c r="Z66" s="4"/>
       <c r="AA66" s="1"/>
       <c r="AB66" s="1"/>
-      <c r="AC66" s="50"/>
+      <c r="AC66" s="38"/>
     </row>
     <row r="67" spans="1:29" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A67" s="54" t="s">
+      <c r="A67" s="40" t="s">
         <v>50</v>
       </c>
-      <c r="B67" s="28" t="s">
+      <c r="B67" s="25" t="s">
         <v>33</v>
       </c>
       <c r="C67" s="2"/>
@@ -3709,13 +3734,13 @@
       <c r="Z67" s="2"/>
       <c r="AA67" s="2"/>
       <c r="AB67" s="1"/>
-      <c r="AC67" s="50"/>
+      <c r="AC67" s="38"/>
     </row>
     <row r="68" spans="1:29" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A68" s="55" t="s">
+      <c r="A68" s="41" t="s">
         <v>109</v>
       </c>
-      <c r="B68" s="30" t="s">
+      <c r="B68" s="27" t="s">
         <v>39</v>
       </c>
       <c r="C68" s="4"/>
@@ -3744,13 +3769,13 @@
       <c r="Z68" s="4"/>
       <c r="AA68" s="4"/>
       <c r="AB68" s="1"/>
-      <c r="AC68" s="50"/>
+      <c r="AC68" s="38"/>
     </row>
     <row r="69" spans="1:29" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A69" s="54" t="s">
+      <c r="A69" s="40" t="s">
         <v>110</v>
       </c>
-      <c r="B69" s="29" t="s">
+      <c r="B69" s="26" t="s">
         <v>34</v>
       </c>
       <c r="C69" s="2"/>
@@ -3779,13 +3804,13 @@
       <c r="Z69" s="2"/>
       <c r="AA69" s="2"/>
       <c r="AB69" s="1"/>
-      <c r="AC69" s="57"/>
+      <c r="AC69" s="42"/>
     </row>
     <row r="70" spans="1:29" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A70" s="55" t="s">
+      <c r="A70" s="41" t="s">
         <v>111</v>
       </c>
-      <c r="B70" s="23" t="s">
+      <c r="B70" s="20" t="s">
         <v>33</v>
       </c>
       <c r="C70" s="4"/>
@@ -3814,45 +3839,45 @@
       <c r="Z70" s="4"/>
       <c r="AA70" s="4"/>
       <c r="AB70" s="4"/>
-      <c r="AC70" s="62"/>
+      <c r="AC70" s="45"/>
     </row>
     <row r="71" spans="1:29" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A71" s="63" t="s">
+      <c r="A71" s="46" t="s">
         <v>51</v>
       </c>
-      <c r="B71" s="64" t="s">
+      <c r="B71" s="47" t="s">
         <v>34</v>
       </c>
-      <c r="C71" s="65"/>
-      <c r="D71" s="65"/>
-      <c r="E71" s="65"/>
-      <c r="F71" s="65"/>
-      <c r="G71" s="65"/>
-      <c r="H71" s="66"/>
-      <c r="I71" s="66"/>
-      <c r="J71" s="65"/>
-      <c r="K71" s="65"/>
-      <c r="L71" s="65"/>
-      <c r="M71" s="65"/>
-      <c r="N71" s="65"/>
-      <c r="O71" s="66"/>
-      <c r="P71" s="66"/>
-      <c r="Q71" s="65"/>
-      <c r="R71" s="65"/>
-      <c r="S71" s="65"/>
-      <c r="T71" s="65"/>
-      <c r="U71" s="65"/>
-      <c r="V71" s="66"/>
-      <c r="W71" s="66"/>
-      <c r="X71" s="65"/>
-      <c r="Y71" s="65"/>
-      <c r="Z71" s="65"/>
-      <c r="AA71" s="65"/>
-      <c r="AB71" s="65"/>
-      <c r="AC71" s="67"/>
+      <c r="C71" s="48"/>
+      <c r="D71" s="48"/>
+      <c r="E71" s="48"/>
+      <c r="F71" s="48"/>
+      <c r="G71" s="48"/>
+      <c r="H71" s="49"/>
+      <c r="I71" s="49"/>
+      <c r="J71" s="48"/>
+      <c r="K71" s="48"/>
+      <c r="L71" s="48"/>
+      <c r="M71" s="48"/>
+      <c r="N71" s="48"/>
+      <c r="O71" s="49"/>
+      <c r="P71" s="49"/>
+      <c r="Q71" s="48"/>
+      <c r="R71" s="48"/>
+      <c r="S71" s="48"/>
+      <c r="T71" s="48"/>
+      <c r="U71" s="48"/>
+      <c r="V71" s="49"/>
+      <c r="W71" s="49"/>
+      <c r="X71" s="48"/>
+      <c r="Y71" s="48"/>
+      <c r="Z71" s="48"/>
+      <c r="AA71" s="48"/>
+      <c r="AB71" s="48"/>
+      <c r="AC71" s="50"/>
     </row>
     <row r="73" spans="1:29" x14ac:dyDescent="0.3">
-      <c r="A73" s="14" t="s">
+      <c r="A73" s="12" t="s">
         <v>52</v>
       </c>
       <c r="B73" s="1"/>
@@ -3901,6 +3926,6 @@
     <mergeCell ref="A51:AC51"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" scale="63" fitToHeight="0" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="54" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>